<commit_message>
Update Q5.13_My_ Movie_ App_Test_Cases.xlsx
</commit_message>
<xml_diff>
--- a/Q5.13_My_ Movie_ App_Test_Cases.xlsx
+++ b/Q5.13_My_ Movie_ App_Test_Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinze\JavaScriptFriday\JSAT2\part5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinze\JavaScriptFriday\GitHub-rchumpon\JSAT2-Part4-Part5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2096E8DE-6F94-4250-A73D-A7AB97DD3ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E3A1B4-F979-42A0-A631-7051DC228525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="617" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -763,6 +763,28 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -775,23 +797,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -809,22 +819,81 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -845,75 +914,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1212,25 +1212,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="20"/>
+      <c r="B1" s="25"/>
       <c r="C1" s="9">
         <v>1</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="20"/>
-      <c r="F1" s="21" t="s">
+      <c r="E1" s="25"/>
+      <c r="F1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2"/>
@@ -1246,101 +1246,101 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="24"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="26">
+      <c r="E3" s="28"/>
+      <c r="F3" s="30">
         <v>45982</v>
       </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="23" t="s">
+      <c r="G3" s="31"/>
+      <c r="H3" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="24"/>
-      <c r="J3" s="12" t="s">
+      <c r="I3" s="28"/>
+      <c r="J3" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="13"/>
+      <c r="K3" s="21"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="29" t="s">
+      <c r="C5" s="23"/>
+      <c r="D5" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="30"/>
-      <c r="F5" s="14" t="s">
+      <c r="E5" s="15"/>
+      <c r="F5" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="14" t="s">
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
     </row>
     <row r="6" spans="1:11" ht="26.5" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
     </row>
     <row r="7" spans="1:11" ht="74.5" customHeight="1">
       <c r="A7" s="4">
         <v>1</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="21" t="s">
+      <c r="C7" s="26"/>
+      <c r="D7" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="21"/>
-      <c r="F7" s="16" t="s">
+      <c r="E7" s="12"/>
+      <c r="F7" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="17"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="17"/>
-      <c r="K7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="18"/>
+      <c r="K7" s="19"/>
     </row>
     <row r="8" spans="1:11" ht="37" customHeight="1">
       <c r="A8" s="4"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="18"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="19"/>
     </row>
     <row r="18" spans="1:1" ht="23.15" customHeight="1"/>
     <row r="19" spans="1:1" ht="68.150000000000006" hidden="1" customHeight="1"/>
@@ -1362,11 +1362,6 @@
     <row r="47" ht="36" customHeight="1"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="F8:H8"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="I5:K6"/>
     <mergeCell ref="I8:K8"/>
@@ -1383,6 +1378,11 @@
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="F5:H6"/>
     <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="F8:H8"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1402,25 +1402,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>10</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>99</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -1436,29 +1436,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -1474,135 +1474,148 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="64" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>101</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="71" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="80" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>82</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="99" customHeight="1">
       <c r="A10" s="11">
         <v>4</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32" t="s">
+      <c r="C10" s="49"/>
+      <c r="D10" s="47" t="s">
         <v>83</v>
       </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34" t="s">
+      <c r="E10" s="49"/>
+      <c r="F10" s="57" t="s">
         <v>84</v>
       </c>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40" t="s">
-        <v>10</v>
-      </c>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:H6"/>
     <mergeCell ref="I5:K6"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
@@ -1619,19 +1632,6 @@
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -1658,25 +1658,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="20"/>
+      <c r="B1" s="25"/>
       <c r="C1" s="9">
         <v>2</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="20"/>
-      <c r="F1" s="21" t="s">
+      <c r="E1" s="25"/>
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2"/>
@@ -1692,111 +1692,111 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="24"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="26">
+      <c r="E3" s="28"/>
+      <c r="F3" s="30">
         <v>45982</v>
       </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="23" t="s">
+      <c r="G3" s="31"/>
+      <c r="H3" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="24"/>
-      <c r="J3" s="12" t="s">
+      <c r="I3" s="28"/>
+      <c r="J3" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="13"/>
+      <c r="K3" s="21"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="29" t="s">
+      <c r="C5" s="23"/>
+      <c r="D5" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="30"/>
-      <c r="F5" s="14" t="s">
+      <c r="E5" s="15"/>
+      <c r="F5" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="14" t="s">
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="15"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
     </row>
     <row r="7" spans="1:11" ht="54" customHeight="1">
       <c r="A7" s="4">
         <v>1</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="21" t="s">
+      <c r="C7" s="26"/>
+      <c r="D7" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="21"/>
-      <c r="F7" s="16" t="s">
+      <c r="E7" s="12"/>
+      <c r="F7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="17"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="17"/>
-      <c r="K7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="18"/>
+      <c r="K7" s="19"/>
     </row>
     <row r="8" spans="1:11" ht="59" customHeight="1">
       <c r="A8" s="4">
         <v>2</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="21" t="s">
+      <c r="C8" s="13"/>
+      <c r="D8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="21"/>
-      <c r="F8" s="16" t="s">
+      <c r="E8" s="12"/>
+      <c r="F8" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="17"/>
-      <c r="K8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="18"/>
+      <c r="K8" s="19"/>
     </row>
     <row r="18" spans="1:1" ht="23.15" customHeight="1"/>
     <row r="19" spans="1:1" ht="68.150000000000006" hidden="1" customHeight="1"/>
@@ -1818,14 +1818,6 @@
     <row r="47" ht="36" customHeight="1"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="F8:H8"/>
@@ -1839,6 +1831,14 @@
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -1857,25 +1857,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>3</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -1891,29 +1891,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -1929,135 +1929,151 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="64" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="71" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>89</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="62.5" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="64" customHeight="1">
       <c r="A10" s="11">
         <v>4</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32" t="s">
+      <c r="C10" s="49"/>
+      <c r="D10" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34" t="s">
+      <c r="E10" s="49"/>
+      <c r="F10" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40" t="s">
-        <v>10</v>
-      </c>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="I7:K7"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:C6"/>
     <mergeCell ref="D5:E6"/>
@@ -2071,22 +2087,6 @@
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="I5:K6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="I10:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2104,25 +2104,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>4</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -2138,29 +2138,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -2176,138 +2176,125 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="64" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>92</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="71" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="62.5" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="64" customHeight="1">
       <c r="A10" s="11"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:H6"/>
-    <mergeCell ref="I5:K6"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
@@ -2324,6 +2311,19 @@
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="I5:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2345,25 +2345,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>5</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -2379,29 +2379,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -2417,148 +2417,135 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="123.5" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>94</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="118.5" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="78.5" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>98</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="64" customHeight="1">
       <c r="A10" s="11">
         <v>4</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="47" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32" t="s">
+      <c r="C10" s="49"/>
+      <c r="D10" s="47" t="s">
         <v>107</v>
       </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34" t="s">
+      <c r="E10" s="49"/>
+      <c r="F10" s="57" t="s">
         <v>108</v>
       </c>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40" t="s">
-        <v>10</v>
-      </c>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:H6"/>
-    <mergeCell ref="I5:K6"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
@@ -2575,6 +2562,19 @@
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="I5:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2595,25 +2595,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>6</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -2629,29 +2629,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -2667,138 +2667,125 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="108.5" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="88.5" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>45</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="78.5" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="64" customHeight="1">
       <c r="A10" s="11"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:H6"/>
-    <mergeCell ref="I5:K6"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
@@ -2815,6 +2802,19 @@
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="I5:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2835,25 +2835,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>7</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -2869,29 +2869,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -2907,138 +2907,125 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="108.5" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="88.5" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="78.5" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="64" customHeight="1">
       <c r="A10" s="11"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:H6"/>
-    <mergeCell ref="I5:K6"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
@@ -3055,6 +3042,19 @@
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="I5:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -3075,25 +3075,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>8</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -3109,29 +3109,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -3147,138 +3147,125 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="108.5" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="88.5" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="78.5" customHeight="1">
       <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="49"/>
+      <c r="D9" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="38"/>
-      <c r="K9" s="39"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="61"/>
+      <c r="K9" s="62"/>
     </row>
     <row r="10" spans="1:11" ht="64" customHeight="1">
       <c r="A10" s="11"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:H6"/>
-    <mergeCell ref="I5:K6"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="D10:E10"/>
@@ -3295,6 +3282,19 @@
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="I5:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -3315,25 +3315,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="10">
         <v>9</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="32" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="47" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="33"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
       <c r="A2" s="6"/>
@@ -3349,29 +3349,29 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="60">
+      <c r="E3" s="51"/>
+      <c r="F3" s="53">
         <v>45982</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="59" t="s">
+      <c r="G3" s="54"/>
+      <c r="H3" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="58"/>
-      <c r="J3" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="63"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="56"/>
     </row>
     <row r="4" spans="1:11" ht="15.5">
       <c r="A4" s="5"/>
@@ -3387,102 +3387,114 @@
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="19" customHeight="1">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="47" t="s">
+      <c r="C5" s="35"/>
+      <c r="D5" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="39"/>
+      <c r="F5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="43" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="51"/>
-      <c r="K5" s="44"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="35"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="42"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="46"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="37"/>
     </row>
     <row r="7" spans="1:11" ht="108.5" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="32" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="49"/>
+      <c r="F7" s="57" t="s">
         <v>75</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
     </row>
     <row r="8" spans="1:11" ht="88.5" customHeight="1">
       <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="47" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="32" t="s">
+      <c r="C8" s="49"/>
+      <c r="D8" s="47" t="s">
         <v>76</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34" t="s">
+      <c r="E8" s="49"/>
+      <c r="F8" s="57" t="s">
         <v>74</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="39"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="61"/>
+      <c r="K8" s="62"/>
     </row>
     <row r="9" spans="1:11" ht="64" customHeight="1">
       <c r="A9" s="11"/>
-      <c r="B9" s="32"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="40"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="36"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="63"/>
+      <c r="J9" s="58"/>
+      <c r="K9" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:K8"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:C6"/>
     <mergeCell ref="D5:E6"/>
@@ -3496,18 +3508,6 @@
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="I5:K6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="I8:K8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>